<commit_message>
nuc abs lim removed; gas buildrate relaxed
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan10/SuppXLS/Scen_Par-AR6_R10.xlsx
+++ b/VerveStacks_IND_grids_kan10/SuppXLS/Scen_Par-AR6_R10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan10\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1CEE6C-2B30-48B3-91B4-91D0F6D49FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE7092F-A31A-47DC-BF4B-51B2F2BB7CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -517,7 +517,7 @@
     <t>aggregators,grid</t>
   </si>
   <si>
-    <t>33-40</t>
+    <t>1-40</t>
   </si>
 </sst>
 </file>
@@ -6109,7 +6109,7 @@
     <row r="2" spans="1:41" x14ac:dyDescent="0.45">
       <c r="D2" s="1" t="str">
         <f>"~Inputcell: "&amp;_xlfn.TEXTJOIN(",",TRUE,I1:EG1)</f>
-        <v>~Inputcell: 33-40</v>
+        <v>~Inputcell: 1-40</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>26</v>

</xml_diff>